<commit_message>
Add Week 11 documentation and timesheet, correct booked hours and remove templates
</commit_message>
<xml_diff>
--- a/Documentation/Week 11/Booked Hours/Booked_Hours_Dhava.xlsx
+++ b/Documentation/Week 11/Booked Hours/Booked_Hours_Dhava.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
   <workbookPr date1904="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wikha\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECB33847-61D1-4F51-BF7E-BB4E92B5B6E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{94337B32-1717-4463-91C6-46362315A3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,38 +17,28 @@
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="25">
-  <si>
-    <t>Wk</t>
-  </si>
-  <si>
-    <t>Begin</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Time</t>
-  </si>
-  <si>
-    <t>End</t>
-  </si>
-  <si>
-    <t>Activity</t>
-  </si>
-  <si>
-    <t>Total
-Hours</t>
-  </si>
-  <si>
-    <t>Session
-Hours</t>
-  </si>
   <si>
     <r>
       <t>CITS3200 Project Billed Hours Record for &lt;Dhava Wikhananda Adhi&gt;</t>
@@ -62,6 +52,32 @@
       <t xml:space="preserve">
 Each time you do some work on the project, note the week number, start and end date and hour, plus a brief description of the activity. At the end of each week send a copy of the sheet as it currently stands to your group's manager for recording on the group TimeSheet. Date in the form DD/MM/YY and time as XX:YY (24hr clock)</t>
     </r>
+  </si>
+  <si>
+    <t>Wk</t>
+  </si>
+  <si>
+    <t>Begin</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>Activity</t>
+  </si>
+  <si>
+    <t>Session
+Hours</t>
+  </si>
+  <si>
+    <t>Total
+Hours</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Time</t>
   </si>
   <si>
     <t>Team meeting</t>
@@ -116,7 +132,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Verdana"/>
@@ -785,23 +801,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I132"/>
-  <sheetFormatPr defaultColWidth="10.6328125" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.625" defaultRowHeight="12.6"/>
   <cols>
-    <col min="1" max="1" width="5.81640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.08984375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.1796875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6328125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="8.81640625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="46.453125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.36328125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.6328125" style="1"/>
-    <col min="9" max="9" width="10.6328125" style="1" hidden="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.6328125" style="1"/>
+    <col min="1" max="1" width="5.875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="46.5" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9.375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="10.625" style="1"/>
+    <col min="9" max="9" width="10.625" style="1" hidden="1" customWidth="1"/>
+    <col min="10" max="16384" width="10.625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="70.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="70.900000000000006" customHeight="1">
       <c r="A1" s="10" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -811,47 +827,47 @@
       <c r="G1" s="11"/>
       <c r="H1" s="12"/>
     </row>
-    <row r="2" spans="1:9" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="16.149999999999999" customHeight="1">
       <c r="A2" s="8" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="16"/>
       <c r="D2" s="15" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2" s="16"/>
       <c r="F2" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="8" t="s">
         <v>5</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>7</v>
       </c>
       <c r="H2" s="13" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="13.05" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="13.15" customHeight="1">
       <c r="A3" s="9"/>
       <c r="B3" s="2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F3" s="18"/>
       <c r="G3" s="9"/>
       <c r="H3" s="14"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -881,7 +897,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9">
       <c r="A5" s="1">
         <v>2</v>
       </c>
@@ -913,7 +929,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9">
       <c r="A6" s="1">
         <v>3</v>
       </c>
@@ -944,7 +960,7 @@
         <v>1.0000000001164153</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9">
       <c r="A7" s="1">
         <v>3</v>
       </c>
@@ -975,7 +991,7 @@
         <v>1.0000000001164153</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9">
       <c r="A8" s="1">
         <v>3</v>
       </c>
@@ -1007,7 +1023,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9">
       <c r="A9" s="1">
         <v>4</v>
       </c>
@@ -1039,7 +1055,7 @@
         <v>1.0000000001164153</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9">
       <c r="A10" s="1">
         <v>4</v>
       </c>
@@ -1071,7 +1087,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9">
       <c r="A11" s="1">
         <v>4</v>
       </c>
@@ -1103,7 +1119,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9">
       <c r="A12" s="1">
         <v>5</v>
       </c>
@@ -1135,7 +1151,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9">
       <c r="A13" s="1">
         <v>5</v>
       </c>
@@ -1167,7 +1183,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9">
       <c r="A14" s="1">
         <v>5</v>
       </c>
@@ -1199,7 +1215,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9">
       <c r="A15" s="1">
         <v>6</v>
       </c>
@@ -1231,7 +1247,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9">
       <c r="A16" s="1">
         <v>6</v>
       </c>
@@ -1263,7 +1279,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9">
       <c r="A17" s="1">
         <v>6</v>
       </c>
@@ -1295,7 +1311,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9">
       <c r="A18" s="1">
         <v>7</v>
       </c>
@@ -1327,7 +1343,7 @@
         <v>9.9999999999417923</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9">
       <c r="A19" s="1">
         <v>7</v>
       </c>
@@ -1359,7 +1375,7 @@
         <v>0.8333333334303461</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9">
       <c r="A20" s="1">
         <v>8</v>
       </c>
@@ -1391,7 +1407,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9">
       <c r="A21" s="1">
         <v>8</v>
       </c>
@@ -1423,7 +1439,7 @@
         <v>1.0000000001164153</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9">
       <c r="A22" s="1">
         <v>8</v>
       </c>
@@ -1455,7 +1471,7 @@
         <v>0.16666666668606922</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9">
       <c r="A23" s="1">
         <v>9</v>
       </c>
@@ -1487,7 +1503,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9">
       <c r="A24" s="1">
         <v>9</v>
       </c>
@@ -1519,7 +1535,7 @@
         <v>1.0000000001164153</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9">
       <c r="A25" s="1">
         <v>9</v>
       </c>
@@ -1551,7 +1567,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9">
       <c r="A26" s="1">
         <v>9</v>
       </c>
@@ -1583,7 +1599,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9">
       <c r="A27" s="1">
         <v>10</v>
       </c>
@@ -1615,7 +1631,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9">
       <c r="A28" s="1">
         <v>10</v>
       </c>
@@ -1647,7 +1663,7 @@
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9">
       <c r="A29" s="1">
         <v>10</v>
       </c>
@@ -1655,7 +1671,7 @@
         <v>44836</v>
       </c>
       <c r="C29" s="5">
-        <v>0.47916666666666669</v>
+        <v>0.97916666666666663</v>
       </c>
       <c r="D29" s="4">
         <v>44837</v>
@@ -1668,18 +1684,18 @@
       </c>
       <c r="G29" s="6">
         <f t="shared" si="0"/>
-        <v>13.000000000116415</v>
+        <v>1.0000000001164153</v>
       </c>
       <c r="H29" s="1">
         <f t="shared" si="2"/>
-        <v>51.499999999825377</v>
+        <v>39.499999999825377</v>
       </c>
       <c r="I29" s="1">
         <f t="shared" si="1"/>
-        <v>13.000000000116415</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+        <v>1.0000000001164153</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
       <c r="A30" s="1">
         <v>11</v>
       </c>
@@ -1704,30 +1720,30 @@
       </c>
       <c r="H30" s="1">
         <f t="shared" si="2"/>
-        <v>51.999999999708962</v>
+        <v>39.999999999708962</v>
       </c>
       <c r="I30" s="1">
         <f t="shared" si="1"/>
         <v>0.49999999988358468</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" ht="15">
       <c r="A31" s="8" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C31" s="16"/>
       <c r="D31" s="15" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E31" s="16"/>
       <c r="F31" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G31" s="7" t="s">
         <v>5</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>7</v>
       </c>
       <c r="H31" s="7" t="s">
         <v>6</v>
@@ -1737,19 +1753,19 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" ht="15">
       <c r="A32" s="9"/>
       <c r="B32" s="2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F32" s="7"/>
       <c r="G32" s="7"/>
@@ -1759,7 +1775,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9">
       <c r="A33" s="1">
         <v>11</v>
       </c>
@@ -1784,14 +1800,14 @@
       </c>
       <c r="H33" s="1">
         <f>IF(AND(G33&lt;&gt;" ",G33&lt;&gt;"ERROR",H30&lt;&gt;" ", H30&lt;&gt;"ERROR"),G33+H30," ")</f>
-        <v>55.499999999767169</v>
+        <v>43.499999999767169</v>
       </c>
       <c r="I33" s="1">
         <f t="shared" si="1"/>
         <v>3.5000000000582077</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9">
       <c r="A34" s="1">
         <v>11</v>
       </c>
@@ -1816,14 +1832,14 @@
       </c>
       <c r="H34" s="1">
         <f t="shared" ref="H34:H64" si="4">IF(AND(G34&lt;&gt;" ",G34&lt;&gt;"ERROR",H33&lt;&gt;" ", H33&lt;&gt;"ERROR"),G34+H33," ")</f>
-        <v>55.999999999650754</v>
+        <v>43.999999999650754</v>
       </c>
       <c r="I34" s="1">
         <f t="shared" si="1"/>
         <v>0.49999999988358468</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9">
       <c r="A35" s="1">
         <v>11</v>
       </c>
@@ -1848,14 +1864,14 @@
       </c>
       <c r="H35" s="1">
         <f t="shared" si="4"/>
-        <v>56.999999999592546</v>
+        <v>44.999999999592546</v>
       </c>
       <c r="I35" s="1">
         <f t="shared" si="1"/>
         <v>0.99999999994179234</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9">
       <c r="A36" s="1">
         <v>11</v>
       </c>
@@ -1880,14 +1896,14 @@
       </c>
       <c r="H36" s="1">
         <f t="shared" si="4"/>
-        <v>57.499999999650754</v>
+        <v>45.499999999650754</v>
       </c>
       <c r="I36" s="1">
         <f t="shared" si="1"/>
         <v>0.50000000005820766</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9">
       <c r="B37" s="4"/>
       <c r="C37" s="5"/>
       <c r="D37" s="4"/>
@@ -1905,7 +1921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9">
       <c r="B38" s="4"/>
       <c r="C38" s="5"/>
       <c r="D38" s="4"/>
@@ -1923,7 +1939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9">
       <c r="B39" s="4"/>
       <c r="C39" s="5"/>
       <c r="D39" s="4"/>
@@ -1941,7 +1957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9">
       <c r="B40" s="4"/>
       <c r="C40" s="5"/>
       <c r="D40" s="4"/>
@@ -1959,7 +1975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9">
       <c r="B41" s="4"/>
       <c r="C41" s="5"/>
       <c r="D41" s="4"/>
@@ -1977,7 +1993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9">
       <c r="B42" s="4"/>
       <c r="C42" s="5"/>
       <c r="D42" s="4"/>
@@ -1995,7 +2011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9">
       <c r="B43" s="4"/>
       <c r="C43" s="5"/>
       <c r="D43" s="4"/>
@@ -2013,7 +2029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9">
       <c r="B44" s="4"/>
       <c r="C44" s="5"/>
       <c r="D44" s="4"/>
@@ -2031,7 +2047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9">
       <c r="B45" s="4"/>
       <c r="C45" s="5"/>
       <c r="D45" s="4"/>
@@ -2049,7 +2065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9">
       <c r="B46" s="4"/>
       <c r="C46" s="5"/>
       <c r="D46" s="4"/>
@@ -2067,7 +2083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9">
       <c r="B47" s="4"/>
       <c r="C47" s="5"/>
       <c r="D47" s="4"/>
@@ -2085,7 +2101,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9">
       <c r="B48" s="4"/>
       <c r="C48" s="5"/>
       <c r="D48" s="4"/>
@@ -2103,7 +2119,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:9">
       <c r="B49" s="4"/>
       <c r="C49" s="5"/>
       <c r="D49" s="4"/>
@@ -2121,7 +2137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:9">
       <c r="B50" s="4"/>
       <c r="C50" s="5"/>
       <c r="D50" s="4"/>
@@ -2139,7 +2155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:9">
       <c r="B51" s="4"/>
       <c r="C51" s="5"/>
       <c r="D51" s="4"/>
@@ -2157,7 +2173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:9">
       <c r="B52" s="4"/>
       <c r="C52" s="5"/>
       <c r="D52" s="4"/>
@@ -2175,7 +2191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:9">
       <c r="B53" s="4"/>
       <c r="C53" s="5"/>
       <c r="D53" s="4"/>
@@ -2193,7 +2209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:9">
       <c r="B54" s="4"/>
       <c r="C54" s="5"/>
       <c r="D54" s="4"/>
@@ -2211,7 +2227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:9">
       <c r="B55" s="4"/>
       <c r="C55" s="5"/>
       <c r="D55" s="4"/>
@@ -2229,7 +2245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:9">
       <c r="B56" s="4"/>
       <c r="C56" s="5"/>
       <c r="D56" s="4"/>
@@ -2247,7 +2263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:9">
       <c r="B57" s="4"/>
       <c r="C57" s="5"/>
       <c r="D57" s="4"/>
@@ -2265,7 +2281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:9">
       <c r="B58" s="4"/>
       <c r="C58" s="5"/>
       <c r="D58" s="4"/>
@@ -2283,7 +2299,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:9">
       <c r="B59" s="4"/>
       <c r="C59" s="5"/>
       <c r="D59" s="4"/>
@@ -2301,7 +2317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:9">
       <c r="B60" s="4"/>
       <c r="G60" s="6" t="str">
         <f t="shared" si="3"/>
@@ -2316,7 +2332,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:9">
       <c r="B61" s="4"/>
       <c r="G61" s="6" t="str">
         <f t="shared" si="3"/>
@@ -2331,7 +2347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:9">
       <c r="B62" s="4"/>
       <c r="G62" s="6" t="str">
         <f t="shared" si="3"/>
@@ -2346,7 +2362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:9">
       <c r="B63" s="4"/>
       <c r="G63" s="6" t="str">
         <f t="shared" si="3"/>
@@ -2361,7 +2377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:9">
       <c r="B64" s="4"/>
       <c r="G64" s="6" t="str">
         <f t="shared" si="3"/>
@@ -2376,23 +2392,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" ht="15">
       <c r="A65" s="8" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C65" s="16"/>
       <c r="D65" s="15" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E65" s="16"/>
       <c r="F65" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G65" s="7" t="s">
         <v>5</v>
-      </c>
-      <c r="G65" s="7" t="s">
-        <v>7</v>
       </c>
       <c r="H65" s="7" t="s">
         <v>6</v>
@@ -2402,19 +2418,19 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" ht="15">
       <c r="A66" s="9"/>
       <c r="B66" s="2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F66" s="7"/>
       <c r="G66" s="7"/>
@@ -2424,7 +2440,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:9">
       <c r="G67" s="6" t="str">
         <f t="shared" ref="G67:G98" si="5">IF(I67&gt;0,I67,IF(I67=0, " ", "ERROR"))</f>
         <v xml:space="preserve"> </v>
@@ -2438,7 +2454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:9">
       <c r="G68" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2452,7 +2468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:9">
       <c r="G69" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2466,7 +2482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:9">
       <c r="G70" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2480,7 +2496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:9">
       <c r="G71" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2494,7 +2510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:9">
       <c r="G72" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2508,7 +2524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:9">
       <c r="G73" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2522,7 +2538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:9">
       <c r="G74" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2536,7 +2552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:9">
       <c r="G75" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2550,7 +2566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:9">
       <c r="G76" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2564,7 +2580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:9">
       <c r="G77" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2578,7 +2594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:9">
       <c r="G78" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2592,7 +2608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:9">
       <c r="G79" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2606,7 +2622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:9">
       <c r="G80" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2620,7 +2636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="81" spans="7:9">
       <c r="G81" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2634,7 +2650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="82" spans="7:9">
       <c r="G82" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2648,7 +2664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="83" spans="7:9">
       <c r="G83" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2662,7 +2678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="84" spans="7:9">
       <c r="G84" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2676,7 +2692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="85" spans="7:9">
       <c r="G85" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2690,7 +2706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="86" spans="7:9">
       <c r="G86" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2704,7 +2720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="87" spans="7:9">
       <c r="G87" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2718,7 +2734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="88" spans="7:9">
       <c r="G88" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2732,7 +2748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="89" spans="7:9">
       <c r="G89" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2746,7 +2762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="90" spans="7:9">
       <c r="G90" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2760,7 +2776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="91" spans="7:9">
       <c r="G91" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2774,7 +2790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="92" spans="7:9">
       <c r="G92" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2788,7 +2804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="93" spans="7:9">
       <c r="G93" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2802,7 +2818,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="94" spans="7:9">
       <c r="G94" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2816,7 +2832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="95" spans="7:9">
       <c r="G95" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2830,7 +2846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="96" spans="7:9">
       <c r="G96" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2844,7 +2860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:9">
       <c r="G97" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2858,7 +2874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:9">
       <c r="G98" s="6" t="str">
         <f t="shared" si="5"/>
         <v xml:space="preserve"> </v>
@@ -2872,23 +2888,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" ht="15">
       <c r="A99" s="8" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B99" s="15" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C99" s="16"/>
       <c r="D99" s="15" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E99" s="16"/>
       <c r="F99" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G99" s="7" t="s">
         <v>5</v>
-      </c>
-      <c r="G99" s="7" t="s">
-        <v>7</v>
       </c>
       <c r="H99" s="7" t="s">
         <v>6</v>
@@ -2898,19 +2914,19 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="15" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" ht="15">
       <c r="A100" s="9"/>
       <c r="B100" s="2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E100" s="3" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F100" s="7"/>
       <c r="G100" s="7"/>
@@ -2920,7 +2936,7 @@
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:9">
       <c r="G101" s="6" t="str">
         <f t="shared" ref="G101:G132" si="8">IF(I101&gt;0,I101,IF(I101=0, " ", "ERROR"))</f>
         <v xml:space="preserve"> </v>
@@ -2934,7 +2950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:9">
       <c r="G102" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -2948,7 +2964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:9">
       <c r="G103" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -2962,7 +2978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:9">
       <c r="G104" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -2976,7 +2992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:9">
       <c r="G105" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -2990,7 +3006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:9">
       <c r="G106" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3004,7 +3020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:9">
       <c r="G107" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3018,7 +3034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:9">
       <c r="G108" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3032,7 +3048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:9">
       <c r="G109" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3046,7 +3062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:9">
       <c r="G110" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3060,7 +3076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:9">
       <c r="G111" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3074,7 +3090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:9">
       <c r="G112" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3088,7 +3104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="113" spans="7:9">
       <c r="G113" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3102,7 +3118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="114" spans="7:9">
       <c r="G114" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3116,7 +3132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="115" spans="7:9">
       <c r="G115" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3130,7 +3146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="116" spans="7:9">
       <c r="G116" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3144,7 +3160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="117" spans="7:9">
       <c r="G117" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3158,7 +3174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="118" spans="7:9">
       <c r="G118" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3172,7 +3188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="119" spans="7:9">
       <c r="G119" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3186,7 +3202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="120" spans="7:9">
       <c r="G120" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3200,7 +3216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="121" spans="7:9">
       <c r="G121" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3214,7 +3230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="122" spans="7:9">
       <c r="G122" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3228,7 +3244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="123" spans="7:9">
       <c r="G123" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3242,7 +3258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="124" spans="7:9">
       <c r="G124" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3256,7 +3272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="125" spans="7:9">
       <c r="G125" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3270,7 +3286,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="126" spans="7:9">
       <c r="G126" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3284,7 +3300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="127" spans="7:9">
       <c r="G127" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3298,7 +3314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="128" spans="7:9">
       <c r="G128" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3312,7 +3328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="129" spans="7:9">
       <c r="G129" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3326,7 +3342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="130" spans="7:9">
       <c r="G130" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3340,7 +3356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="131" spans="7:9">
       <c r="G131" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3354,7 +3370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="7:9" x14ac:dyDescent="0.2">
+    <row r="132" spans="7:9">
       <c r="G132" s="6" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve"> </v>
@@ -3406,7 +3422,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.6"/>
   <sheetData/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3418,7 +3434,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="12.6" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.875" defaultRowHeight="12.6"/>
   <sheetData/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>